<commit_message>
fix: fixing times sum when more than one page exists
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Sequence Extra Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Sequence Extra Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\job\Supervisor app\Server\SupervisorMobility.API\DataAccess\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C96B233-AB28-4637-A323-7CBA1FA335E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AACA4781-21A9-4B48-88C6-3729D54C038C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="52125" yWindow="6255" windowWidth="24825" windowHeight="12240" xr2:uid="{5C2358AE-3AF7-4E65-B536-0B800FE99199}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{5C2358AE-3AF7-4E65-B536-0B800FE99199}"/>
   </bookViews>
   <sheets>
     <sheet name="Name" sheetId="2" r:id="rId1"/>
@@ -572,68 +572,17 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -647,8 +596,59 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1004,36 +1004,36 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="25" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="15"/>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15"/>
-      <c r="G3" s="15"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="25"/>
+      <c r="F3" s="25"/>
+      <c r="G3" s="25"/>
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:16" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="19"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="24" t="s">
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="17" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="24"/>
-      <c r="J5" s="18" t="s">
+      <c r="I5" s="17"/>
+      <c r="J5" s="28" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="19"/>
-      <c r="L5" s="25"/>
+      <c r="K5" s="29"/>
+      <c r="L5" s="34"/>
       <c r="M5" s="14" t="s">
         <v>8</v>
       </c>
@@ -1042,62 +1042,62 @@
       <c r="P5" s="13"/>
     </row>
     <row r="6" spans="2:16" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="17"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="22"/>
-      <c r="G6" s="23"/>
+      <c r="B6" s="27"/>
+      <c r="C6" s="31"/>
+      <c r="D6" s="32"/>
+      <c r="E6" s="32"/>
+      <c r="F6" s="32"/>
+      <c r="G6" s="33"/>
       <c r="H6" s="12" t="s">
         <v>7</v>
       </c>
       <c r="I6" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="J6" s="21"/>
-      <c r="K6" s="22"/>
-      <c r="L6" s="26"/>
+      <c r="J6" s="31"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="35"/>
     </row>
     <row r="7" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="11"/>
-      <c r="C7" s="29"/>
-      <c r="D7" s="30"/>
-      <c r="E7" s="30"/>
-      <c r="F7" s="30"/>
-      <c r="G7" s="31"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="37"/>
+      <c r="E7" s="37"/>
+      <c r="F7" s="37"/>
+      <c r="G7" s="38"/>
       <c r="H7" s="10"/>
       <c r="I7" s="10"/>
-      <c r="J7" s="29"/>
-      <c r="K7" s="30"/>
-      <c r="L7" s="32"/>
+      <c r="J7" s="36"/>
+      <c r="K7" s="37"/>
+      <c r="L7" s="41"/>
     </row>
     <row r="8" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="9"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
+      <c r="C8" s="39"/>
+      <c r="D8" s="40"/>
+      <c r="E8" s="40"/>
+      <c r="F8" s="40"/>
+      <c r="G8" s="40"/>
       <c r="H8" s="8"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="33"/>
-      <c r="K8" s="34"/>
-      <c r="L8" s="35"/>
+      <c r="J8" s="39"/>
+      <c r="K8" s="40"/>
+      <c r="L8" s="42"/>
     </row>
     <row r="9" spans="2:16" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="37"/>
-      <c r="D9" s="37"/>
-      <c r="E9" s="37"/>
-      <c r="F9" s="37"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="42"/>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="15"/>
       <c r="I9" s="6"/>
-      <c r="J9" s="39"/>
-      <c r="K9" s="40"/>
-      <c r="L9" s="41"/>
+      <c r="J9" s="22"/>
+      <c r="K9" s="23"/>
+      <c r="L9" s="24"/>
     </row>
     <row r="10" spans="2:16" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B10" s="5"/>
@@ -1105,30 +1105,35 @@
       <c r="L10" s="3"/>
     </row>
     <row r="11" spans="2:16" ht="17.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="24"/>
-      <c r="D11" s="24"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="17"/>
       <c r="E11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="28" t="s">
+      <c r="F11" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="G11" s="24"/>
-      <c r="H11" s="24"/>
-      <c r="I11" s="28" t="s">
+      <c r="G11" s="17"/>
+      <c r="H11" s="17"/>
+      <c r="I11" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="J11" s="24"/>
-      <c r="K11" s="24"/>
+      <c r="J11" s="17"/>
+      <c r="K11" s="17"/>
       <c r="L11" s="1" t="s">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:G6"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="J5:L6"/>
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="F11:H11"/>
     <mergeCell ref="I11:K11"/>
@@ -1138,11 +1143,6 @@
     <mergeCell ref="J8:L8"/>
     <mergeCell ref="B9:G9"/>
     <mergeCell ref="J9:L9"/>
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:G6"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="J5:L6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>